<commit_message>
La parola «coorte» viene spiegata la prima volta che compare
</commit_message>
<xml_diff>
--- a/clienti-che-tornano.xlsx
+++ b/clienti-che-tornano.xlsx
@@ -12,10 +12,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrice per calendario" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riacquisto" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valore e pareggio" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dati coorti" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coorti (mese d'ingresso)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Dati coorti'!$A$1:$H$277</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Coorti (mese d''ingresso)'!$A$1:$H$277</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>

</xml_diff>

<commit_message>
Il valore di chi torna senza girare in tondo: gruppo nei primi 90 giorni, spesa dal 91 al 365
Il confronto di prima misurava la spesa dello stesso anno che definiva chi torna.
A parita' di spesa nei primi 90 giorni, essere tornati aggiunge 150 sterline
(IC da -34 a 372): conta il volume, non il ritorno. La soglia di 225 e' ritirata.
Ricontato a parte in 06_ricontrollo.py (68 su 68). Riportata nel modello della
pagina la correzione delle intestazioni, che esisteva solo in index.html.
</commit_message>
<xml_diff>
--- a/clienti-che-tornano.xlsx
+++ b/clienti-che-tornano.xlsx
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:B28"/>
+  <dimension ref="A2:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -609,89 +609,117 @@
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>E LA COSA CHE NON ERA IN PROGRAMMA</t>
+          <t>CORRETTO IL 2 OTTOBRE 2026</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>La retention di questo negozio non e' una curva di abbandono: e' un calendario.</t>
+          <t>Il confronto qui sopra definiva «chi torna» con gli ordini del primo anno e misurava la spesa dello stesso anno: la differenza conteneva gli ordini del ritorno.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Il mese dell'anno spiega il 34.8% della variazione fra le celle, l'eta' del cliente solo il 16.6%. Novembre 25%, gennaio 11%.</t>
+          <t>Rifatto con i primi 90 giorni che decidono il gruppo e la spesa dal giorno 91 al 365: a parita' di primo ordine chi e' tornato spende 756 £ in piu'; a parita' di spesa nei primi 90 giorni solo 150 £ (intervallo -34–372. comprende lo zero).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Leggere la matrice da sinistra a destra vuol dire leggere il Natale e chiamarlo fedelta'. I due fogli «Matrice» mostrano le stesse celle nei due allineamenti: confrontali.</t>
+          <t>Conta il volume, non il ritorno in se'. La soglia del foglio «Valore e pareggio» e' ritirata: resta per mostrare cosa diceva.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="3" t="inlineStr">
         <is>
+          <t>E LA COSA CHE NON ERA IN PROGRAMMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>La retention di questo negozio non e' una curva di abbandono: e' un calendario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Il mese dell'anno spiega il 34.8% della variazione fra le celle, l'eta' del cliente solo il 16.6%. Novembre 25%, gennaio 11%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Leggere la matrice da sinistra a destra vuol dire leggere il Natale e chiamarlo fedelta'. I due fogli «Matrice» mostrano le stesse celle nei due allineamenti: confrontali.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="3" t="inlineStr">
+        <is>
           <t>COSA QUESTI NUMERI NON DICONO</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>• Non dicono se trattenere convenga piu' che acquisire: manca il costo di acquisizione. Dicono a che prezzo le due cose si equivalgono.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>• Misurano ricavo, non profitto: manca il costo del venduto. Il margine e' un parametro dichiarato, non un risultato.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>• Il 22,8% delle righe non ha un identificativo cliente. Il tasso di ritorno vero sta fra il 29.0% e il 72.3%: si scrive «tre clienti IDENTIFICATI su quattro tornano».</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>• Non dimostrano una causa. «I clienti che tornano valgono N volte» e' vero; «farli tornare li fa valere N volte» richiederebbe un esperimento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>• I dati sono del 2009-2011. Il metodo si trasferisce, i numeri no.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>COME E' STATO FATTO</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Python e SQL (MySQL 8, funzioni finestra). Le pulizie, il modello, le verifiche e i limiti stanno nel repo, un documento per ognuno.</t>
+          <t>• Il 22,8% delle righe non ha un identificativo cliente. Il tasso di ritorno vero sta fra il 29.0% e il 72.3%: si scrive «tre clienti IDENTIFICATI su quattro tornano».</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>• Non dimostrano una causa. «I clienti che tornano valgono N volte» e' vero; «farli tornare li fa valere N volte» richiederebbe un esperimento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>• I dati sono del 2009-2011. Il metodo si trasferisce, i numeri no.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>COME E' STATO FATTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Python e SQL (MySQL 8, funzioni finestra). Le pulizie, il modello, le verifiche e i limiti stanno nel repo, un documento per ognuno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Le cifre di questo file escono dallo stesso file di dati della pagina web, e sono ricontrollate da uno script che rifa' 63 conti dalle tabelle di base.</t>
         </is>

</xml_diff>

<commit_message>
README con i soli numeri attuali, le correzioni in CHANGELOG.md, e la lettura predittiva dichiarata
L'appaiamento sulla spesa a 90 giorni contiene gia' il secondo ordine: scritto
che e' una lettura predittiva, non causale. Intervalli ricampionati per cliente
dentro gli strati. Mese basso di riferimento: febbraio (due anni), non gennaio.
</commit_message>
<xml_diff>
--- a/clienti-che-tornano.xlsx
+++ b/clienti-che-tornano.xlsx
@@ -623,14 +623,14 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Rifatto con i primi 90 giorni che decidono il gruppo e la spesa dal giorno 91 al 365: a parita' di primo ordine chi e' tornato spende 756 £ in piu'; a parita' di spesa nei primi 90 giorni solo 150 £ (intervallo -34–372. comprende lo zero).</t>
+          <t>Rifatto con i primi 90 giorni che decidono il gruppo e la spesa dal giorno 91 al 365: a parita' di primo ordine chi e' tornato spende 756 £ in piu'; a parita' di spesa nei primi 90 giorni solo 150 £ (intervallo -67–374. comprende lo zero).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Conta il volume, non il ritorno in se'. La soglia del foglio «Valore e pareggio» e' ritirata: resta per mostrare cosa diceva.</t>
+          <t>Per prevedere la spesa futura basta la spesa iniziale (lettura predittiva, non causale). La soglia del foglio «Valore e pareggio» e' ritirata: resta per mostrare cosa diceva.</t>
         </is>
       </c>
     </row>

</xml_diff>